<commit_message>
Suite TD: organizzazione finale aggiornata
</commit_message>
<xml_diff>
--- a/docs/SuiteTD_organigramma_TD.xlsx
+++ b/docs/SuiteTD_organigramma_TD.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -529,13 +529,11 @@
           <t>Toscana Diagnostica</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>DIREZIONE</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Chief Executive Officer</t>
@@ -546,7 +544,6 @@
           <t>Epifani Francesco</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>SI</t>
@@ -564,13 +561,11 @@
           <t>Toscana Diagnostica</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>DIREZIONE</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Chief Operating Officer</t>
@@ -581,7 +576,6 @@
           <t>Zezza Valentina</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>NO</t>
@@ -599,13 +593,11 @@
           <t>Toscana Diagnostica</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>DIREZIONE</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>Chief Financial Officer</t>
@@ -616,7 +608,6 @@
           <t>Malenchini Vincenzo</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>NO</t>
@@ -634,13 +625,11 @@
           <t>Toscana Diagnostica</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>DIREZIONE</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>Chief of Legal, People and Organization</t>
@@ -651,7 +640,6 @@
           <t>Corradi Angelica</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>NO</t>
@@ -669,13 +657,11 @@
           <t>Toscana Diagnostica</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>DIREZIONE</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>Flow &amp; Back Office Management</t>
@@ -686,7 +672,6 @@
           <t>Greco Rosetta</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>NO</t>
@@ -704,13 +689,11 @@
           <t>Toscana Diagnostica</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>DIREZIONE</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>Retail &amp; Communications Management</t>
@@ -721,7 +704,6 @@
           <t>Sansoni Silvia</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>NO</t>
@@ -739,13 +721,11 @@
           <t>Toscana Diagnostica</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>DIREZIONE</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>HSQ Management</t>
@@ -756,7 +736,6 @@
           <t>Cupelli Iacopo</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>NO</t>
@@ -784,7 +763,6 @@
           <t>AREA</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>Responsabile di area</t>
@@ -795,7 +773,6 @@
           <t>Zezza Valentina</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>SI</t>
@@ -823,7 +800,6 @@
           <t>AREA</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>Direttore Tecnico</t>
@@ -834,7 +810,6 @@
           <t>Balzano Maria Teresa</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>NO</t>
@@ -862,7 +837,6 @@
           <t>AREA</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>Direttore Sanitario</t>
@@ -873,7 +847,6 @@
           <t>Taddei Gian Luigi</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>NO</t>
@@ -901,7 +874,6 @@
           <t>AREA</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>Lab Operations Manager</t>
@@ -912,7 +884,6 @@
           <t>Arrighetti Sara</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>NO</t>
@@ -940,7 +911,6 @@
           <t>AREA</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>Responsabile di area</t>
@@ -951,7 +921,6 @@
           <t>Sansoni Silvia</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>SI</t>
@@ -979,7 +948,6 @@
           <t>AREA</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>Responsabile di area</t>
@@ -990,7 +958,6 @@
           <t>Epifani Francesco</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1018,7 +985,6 @@
           <t>AREA</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>Responsabile di area</t>
@@ -1029,7 +995,6 @@
           <t>Greco Rosetta</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1057,7 +1022,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>Site Manager</t>
@@ -1068,7 +1032,6 @@
           <t>De Marco Angela</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1096,7 +1059,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>Direttore Sanitario</t>
@@ -1107,7 +1069,6 @@
           <t>Saltarelli Oreste</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1135,7 +1096,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>Site Manager</t>
@@ -1146,7 +1106,6 @@
           <t>Gabellini Riccardo</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1174,7 +1133,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>Direttore Sanitario</t>
@@ -1185,7 +1143,6 @@
           <t>Gastaldi Roberto</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1213,7 +1170,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>Direttore Sanitario</t>
@@ -1224,7 +1180,6 @@
           <t>Chiaverini Alessandro</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1252,11 +1207,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>3</t>
@@ -1279,7 +1229,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>Direttore Sanitario</t>
@@ -1290,7 +1239,6 @@
           <t>Chiaverini Alessandro</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1318,11 +1266,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>4</t>
@@ -1345,7 +1288,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>Direttore Sanitario</t>
@@ -1356,7 +1298,6 @@
           <t>Chiaverini Alessandro</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1384,11 +1325,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>5</t>
@@ -1411,7 +1347,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>Site Manager</t>
@@ -1422,7 +1357,6 @@
           <t>Mucci Piera</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1450,7 +1384,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>Direttore Sanitario</t>
@@ -1461,7 +1394,6 @@
           <t>Taddei Gian Luigi</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1489,7 +1421,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>Site Manager</t>
@@ -1500,7 +1431,6 @@
           <t>Gelli Manuela</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1528,7 +1458,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>Direttore Sanitario</t>
@@ -1539,7 +1468,6 @@
           <t>Taddei Gian Luigi</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1567,7 +1495,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>Site Manager</t>
@@ -1578,7 +1505,6 @@
           <t>Gucci Lorenzo</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1606,7 +1532,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>Direttore Sanitario</t>
@@ -1617,7 +1542,6 @@
           <t>Taddei Gian Luigi</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1645,7 +1569,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>Site Manager</t>
@@ -1656,7 +1579,6 @@
           <t>Monti Milena</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1684,7 +1606,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>Direttore Sanitario</t>
@@ -1695,7 +1616,6 @@
           <t>Taddei Gian Luigi</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1723,7 +1643,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>Direttore Sanitario</t>
@@ -1734,7 +1653,6 @@
           <t>Taddei Gian Luigi</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1762,11 +1680,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>5</t>
@@ -1789,7 +1702,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>Direttore Sanitario</t>
@@ -1800,7 +1712,6 @@
           <t>Taddei Gian Luigi</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1828,11 +1739,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>6</t>
@@ -1855,7 +1761,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>Direttore Sanitario</t>
@@ -1866,7 +1771,6 @@
           <t>Taddei Gian Luigi</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1894,11 +1798,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
           <t>7</t>
@@ -1921,7 +1820,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>Direttore Sanitario</t>
@@ -1932,7 +1830,6 @@
           <t>Taddei Gian Luigi</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1960,11 +1857,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
           <t>8</t>
@@ -1987,7 +1879,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>Direttore Sanitario</t>
@@ -1998,7 +1889,6 @@
           <t>Taddei Gian Luigi</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>NO</t>
@@ -2026,11 +1916,6 @@
           <t>SEDE</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
           <t>9</t>
@@ -2053,7 +1938,6 @@
           <t>FUNZIONE</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>Responsabile</t>
@@ -2064,7 +1948,6 @@
           <t>Greco Rosetta</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>SI</t>
@@ -2092,7 +1975,6 @@
           <t>FUNZIONE</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>Responsabile</t>
@@ -2103,7 +1985,6 @@
           <t>Corradi Angelica</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>SI</t>
@@ -2131,7 +2012,6 @@
           <t>FUNZIONE</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>Responsabile</t>
@@ -2142,7 +2022,6 @@
           <t>Cesati Valentina</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>SI</t>
@@ -2157,7 +2036,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Preanalitica</t>
+          <t>Laboratorio Sesto Fiorentino</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2167,18 +2046,18 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>REPARTO</t>
+          <t>SEDE</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Responsabile di reparto</t>
+          <t>Direttore Tecnico</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Arrighetti Sara</t>
+          <t>Balzano Maria Teresa</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
@@ -2196,7 +2075,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Core Lab</t>
+          <t>Laboratorio Sesto Fiorentino</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2206,41 +2085,41 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>REPARTO</t>
+          <t>SEDE</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Responsabile di reparto</t>
+          <t>Direttore Sanitario</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Esposito Antonia</t>
+          <t>Taddei Gian Luigi</t>
         </is>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Microbiologia</t>
+          <t>Preanalitica</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Laboratorio di Analisi</t>
+          <t>Laboratorio Sesto Fiorentino</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2248,7 +2127,6 @@
           <t>REPARTO</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
           <t>Responsabile di reparto</t>
@@ -2256,10 +2134,9 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Chilleri Chiara</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr"/>
+          <t>Arrighetti Sara</t>
+        </is>
+      </c>
       <c r="H49" t="inlineStr">
         <is>
           <t>SI</t>
@@ -2267,19 +2144,19 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Biologia Molecolare</t>
+          <t>Core Lab</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Laboratorio di Analisi</t>
+          <t>Laboratorio Sesto Fiorentino</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2287,7 +2164,6 @@
           <t>REPARTO</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t>Responsabile di reparto</t>
@@ -2295,10 +2171,9 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Quattrone Silvia</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr"/>
+          <t>Esposito Antonia</t>
+        </is>
+      </c>
       <c r="H50" t="inlineStr">
         <is>
           <t>SI</t>
@@ -2306,19 +2181,19 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Anatomia Patologica</t>
+          <t>Microbiologia</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Laboratorio di Analisi</t>
+          <t>Laboratorio Sesto Fiorentino</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2326,7 +2201,6 @@
           <t>REPARTO</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>Responsabile di reparto</t>
@@ -2334,10 +2208,9 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Fondi Cristina</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr"/>
+          <t>Chilleri Chiara</t>
+        </is>
+      </c>
       <c r="H51" t="inlineStr">
         <is>
           <t>SI</t>
@@ -2345,44 +2218,116 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>Biologia Molecolare</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Laboratorio Sesto Fiorentino</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>REPARTO</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Responsabile di reparto</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Quattrone Silvia</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>Anatomia Patologica</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Laboratorio di Analisi</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Laboratorio Sesto Fiorentino</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
         <is>
           <t>REPARTO</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr">
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Responsabile di reparto</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Fondi Cristina</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Anatomia Patologica</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Laboratorio Sesto Fiorentino</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>REPARTO</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>Responsabile Tecnico</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>Barelli Stefania</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr">
+      <c r="H54" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="I54" t="inlineStr">
         <is>
           <t>5</t>
         </is>

</xml_diff>